<commit_message>
PipelinePredictRequest.cs  - insert the setting predict cluster output csv
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/Book2.xlsx
+++ b/1.training_model/supplementary/Book2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23EF7F2C-260F-4E59-AF43-64B3A933FF99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94153A9C-3833-40ED-90CB-45EF698D7F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E2D4BE2-B4F1-4052-888A-00209692557E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0E2D4BE2-B4F1-4052-888A-00209692557E}"/>
   </bookViews>
   <sheets>
     <sheet name="Cluster INFO" sheetId="1" r:id="rId1"/>
@@ -100,13 +100,13 @@
     <xdr:from>
       <xdr:col>21</xdr:col>
       <xdr:colOff>495086</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>140157</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>156182</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>118567</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -177,13 +177,13 @@
     <xdr:from>
       <xdr:col>25</xdr:col>
       <xdr:colOff>156182</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>38648</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>29</xdr:col>
       <xdr:colOff>425996</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>4294</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -233,13 +233,13 @@
     <xdr:from>
       <xdr:col>29</xdr:col>
       <xdr:colOff>425996</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>99301</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>33</xdr:col>
       <xdr:colOff>34248</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>90714</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -314,13 +314,13 @@
     <xdr:from>
       <xdr:col>23</xdr:col>
       <xdr:colOff>391721</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>80065</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
       <xdr:colOff>233034</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>120921</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -369,13 +369,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>544640</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>16008</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>31965</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>145143</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -450,13 +450,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>288303</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>141968</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>297299</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>161567</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -505,15 +505,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>314634</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>164766</xdr:rowOff>
+      <xdr:colOff>253481</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>153308</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>479734</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>108941</xdr:rowOff>
+      <xdr:colOff>424931</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>97483</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -528,8 +528,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13116234" y="2558716"/>
-          <a:ext cx="2603500" cy="312475"/>
+          <a:off x="13124655" y="3068786"/>
+          <a:ext cx="2623102" cy="308610"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -582,15 +582,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>23</xdr:col>
-      <xdr:colOff>325634</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>118567</xdr:rowOff>
+      <xdr:colOff>327222</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>121742</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
-      <xdr:colOff>397184</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>164766</xdr:rowOff>
+      <xdr:colOff>342381</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>153308</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -608,8 +608,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14346434" y="1960067"/>
-          <a:ext cx="71550" cy="598649"/>
+          <a:off x="14424222" y="2490568"/>
+          <a:ext cx="15159" cy="578218"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -639,7 +639,7 @@
     <xdr:from>
       <xdr:col>27</xdr:col>
       <xdr:colOff>198968</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>145263</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="385105" cy="264560"/>
@@ -697,7 +697,7 @@
     <xdr:from>
       <xdr:col>23</xdr:col>
       <xdr:colOff>48386</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>156978</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="346826" cy="264560"/>
@@ -754,15 +754,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>311240</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>153045</xdr:rowOff>
+      <xdr:colOff>248154</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>144762</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>482549</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>47126</xdr:rowOff>
+      <xdr:colOff>419463</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>42018</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -777,8 +777,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13112840" y="3283595"/>
-          <a:ext cx="2609709" cy="446531"/>
+          <a:off x="13119328" y="3789110"/>
+          <a:ext cx="2622961" cy="443908"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -831,15 +831,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>23</xdr:col>
-      <xdr:colOff>396895</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>108941</xdr:rowOff>
+      <xdr:colOff>333809</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>97483</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
-      <xdr:colOff>397184</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>153045</xdr:rowOff>
+      <xdr:colOff>342381</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>141587</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -857,8 +857,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="14417695" y="2871191"/>
-          <a:ext cx="289" cy="412404"/>
+          <a:off x="14430809" y="3377396"/>
+          <a:ext cx="8572" cy="408539"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -888,13 +888,13 @@
     <xdr:from>
       <xdr:col>25</xdr:col>
       <xdr:colOff>156182</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>34222</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>29</xdr:col>
       <xdr:colOff>199701</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>128311</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -943,13 +943,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>135374</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>161567</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>449698</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>105682</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1024,13 +1024,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>237794</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>167743</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>354047</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>110153</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1105,13 +1105,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>297299</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>105682</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>297299</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>164568</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1161,13 +1161,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>354047</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>48234</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>371938</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>60305</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1217,7 +1217,7 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>572123</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>143726</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1004699" cy="264560"/>
@@ -1280,7 +1280,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>165250</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>158230</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1114023" cy="264560"/>
@@ -1343,13 +1343,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>295921</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>110153</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>298618</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>16565</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1398,13 +1398,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>371938</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>15</xdr:row>
       <xdr:rowOff>21967</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>540398</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>98641</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1479,13 +1479,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>47733</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>170389</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>412750</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>89025</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1582,13 +1582,13 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>456168</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>98641</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>230242</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>170389</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1638,13 +1638,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>349537</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>98641</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>456168</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>170391</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1694,13 +1694,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>274183</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>2491</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>187808</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>28</xdr:row>
       <xdr:rowOff>155245</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1822,13 +1822,13 @@
     <xdr:from>
       <xdr:col>13</xdr:col>
       <xdr:colOff>230242</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>89025</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>230996</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>2491</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1878,13 +1878,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>185551</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>170391</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>513522</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>93871</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1994,13 +1994,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>276012</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>92688</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>213645</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>178559</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2102,13 +2102,13 @@
     <xdr:from>
       <xdr:col>13</xdr:col>
       <xdr:colOff>230996</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>28</xdr:row>
       <xdr:rowOff>155245</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>244829</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>92688</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -2158,13 +2158,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>212393</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>9968</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>328646</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>135551</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2227,13 +2227,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>392206</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>112059</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>216820</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>137212</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -2603,12 +2603,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEE72467-C912-4492-A3B4-E8AAA2E9F6A2}">
-  <dimension ref="I15:J15"/>
+  <dimension ref="I18:J18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="15" spans="9:10" x14ac:dyDescent="0.35">
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
+    <row r="18" spans="9:10" x14ac:dyDescent="0.35">
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>